<commit_message>
Corrige migrate:fresh sur PostgreSQL et normalise les emails ANBG
Migration strengthen_db_constraints: verifie l'existence des contraintes avant ADD CONSTRAINT, ce qui evitait l'avortement de transaction PostgreSQL (25P02) bloquant migrate:fresh. Bug invisible en test (SQLite saute la branche pgsql).

Convention email {initiale}.{nom}.anbg@gmail.com appliquee a 3 endroits coherents: seeder (AnbgOrganizationSeeder/SyncOrgUsersPreservingPasswordsSeeder), classeur source .xlsx (75 emails) et fixtures de test (28 references / 8 fichiers). Comptes directeur.*, admin, superadmin, dga, ingrid laisses en @anbg.ga.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/base_utilisateurs_pas_anbg_refaite_nouvelle_logique.xlsx
+++ b/docs/base_utilisateurs_pas_anbg_refaite_nouvelle_logique.xlsx
@@ -69,7 +69,7 @@
     <t>MBAZOGO NGUEMA Suzy</t>
   </si>
   <si>
-    <t>suzy.mbazogo@anbg.ga</t>
+    <t>s.mbazogo.anbg@gmail.com</t>
   </si>
   <si>
     <t>UCAS</t>
@@ -84,7 +84,7 @@
     <t>LEKOSSO Ismene</t>
   </si>
   <si>
-    <t>ismene.lekosso@anbg.ga</t>
+    <t>i.lekosso.anbg@gmail.com</t>
   </si>
   <si>
     <t>Agent</t>
@@ -99,19 +99,19 @@
     <t>MATSOMBI DOGUI Reine</t>
   </si>
   <si>
-    <t>reine.matsombi@anbg.ga</t>
+    <t>r.matsombi.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOUKAMBOU Guy Vincent</t>
   </si>
   <si>
-    <t>guy.moukambou@anbg.ga</t>
+    <t>g.moukambou.anbg@gmail.com</t>
   </si>
   <si>
     <t>OKOUMA Miguelle</t>
   </si>
   <si>
-    <t>miguelle.okouma@anbg.ga</t>
+    <t>m.okouma.anbg@gmail.com</t>
   </si>
   <si>
     <t>Directeur DAF</t>
@@ -132,7 +132,7 @@
     <t>INDENGUELA Aldrich</t>
   </si>
   <si>
-    <t>aldrich.indenguela@anbg.ga</t>
+    <t>a.indenguela.anbg@gmail.com</t>
   </si>
   <si>
     <t>AJARH</t>
@@ -144,7 +144,7 @@
     <t>ENGONE Charles</t>
   </si>
   <si>
-    <t>charles.engone@anbg.ga</t>
+    <t>c.engone.anbg@gmail.com</t>
   </si>
   <si>
     <t>Responsable RH</t>
@@ -156,7 +156,7 @@
     <t>MATTEYA Aicha</t>
   </si>
   <si>
-    <t>aicha.matteya@anbg.ga</t>
+    <t>a.matteya.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chef service</t>
@@ -165,7 +165,7 @@
     <t>NGOMBI Charlaine</t>
   </si>
   <si>
-    <t>charlaine.ngombi@anbg.ga</t>
+    <t>c.ngombi.anbg@gmail.com</t>
   </si>
   <si>
     <t>Responsable juridique</t>
@@ -174,7 +174,7 @@
     <t>MIKODJI Casimir</t>
   </si>
   <si>
-    <t>casimir.mikodji@anbg.ga</t>
+    <t>c.mikodji.anbg@gmail.com</t>
   </si>
   <si>
     <t>AMG</t>
@@ -186,13 +186,13 @@
     <t>NGALIBAMA Grasmy</t>
   </si>
   <si>
-    <t>grasmy.ngalibama@anbg.ga</t>
+    <t>g.ngalibama.anbg@gmail.com</t>
   </si>
   <si>
     <t>NGWELEH Igor</t>
   </si>
   <si>
-    <t>igor.ngweleh@anbg.ga</t>
+    <t>i.ngweleh.anbg@gmail.com</t>
   </si>
   <si>
     <t>Transport</t>
@@ -201,7 +201,7 @@
     <t>AFFANE Saturnin</t>
   </si>
   <si>
-    <t>saturnin.affane@anbg.ga</t>
+    <t>s.affane.anbg@gmail.com</t>
   </si>
   <si>
     <t>Parc auto</t>
@@ -210,7 +210,7 @@
     <t>BINGOUMA Ines</t>
   </si>
   <si>
-    <t>ines.bingouma@anbg.ga</t>
+    <t>i.bingouma.anbg@gmail.com</t>
   </si>
   <si>
     <t>Logistique</t>
@@ -219,13 +219,13 @@
     <t>EYEANG Sonia</t>
   </si>
   <si>
-    <t>sonia.eyeang@anbg.ga</t>
+    <t>s.eyeang.anbg@gmail.com</t>
   </si>
   <si>
     <t>MIKOLO Ulrich</t>
   </si>
   <si>
-    <t>ulrich.mikolo@anbg.ga</t>
+    <t>u.mikolo.anbg@gmail.com</t>
   </si>
   <si>
     <t>Responsable voyage</t>
@@ -234,7 +234,7 @@
     <t>ABOGO Melissa</t>
   </si>
   <si>
-    <t>melissa.abogo@anbg.ga</t>
+    <t>m.abogo.anbg@gmail.com</t>
   </si>
   <si>
     <t>SFC</t>
@@ -246,7 +246,7 @@
     <t>MADIBA Herbert</t>
   </si>
   <si>
-    <t>herbert.madiba@anbg.ga</t>
+    <t>h.madiba.anbg@gmail.com</t>
   </si>
   <si>
     <t>Gestionnaire</t>
@@ -255,43 +255,43 @@
     <t>MAPAGA Yannis</t>
   </si>
   <si>
-    <t>yannis.mapaga@anbg.ga</t>
+    <t>y.mapaga.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOUALOUANGO Molan</t>
   </si>
   <si>
-    <t>molan.moualouango@anbg.ga</t>
+    <t>m.moualouango.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOUEBI Yannick</t>
   </si>
   <si>
-    <t>yannick.mouebi@anbg.ga</t>
+    <t>y.mouebi.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOUKONGO Candy</t>
   </si>
   <si>
-    <t>candy.moukongo@anbg.ga</t>
+    <t>c.moukongo.anbg@gmail.com</t>
   </si>
   <si>
     <t>NDAKISSA Tassiana</t>
   </si>
   <si>
-    <t>tassiana.ndakissa@anbg.ga</t>
+    <t>t.ndakissa.anbg@gmail.com</t>
   </si>
   <si>
     <t>EKOMI Robert</t>
   </si>
   <si>
-    <t>robert.ekomi@anbg.ga</t>
+    <t>r.ekomi.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOULOUNGUI Audrey</t>
   </si>
   <si>
-    <t>audrey.mouloungui@anbg.ga</t>
+    <t>a.mouloungui.anbg@gmail.com</t>
   </si>
   <si>
     <t>Suivi administratif</t>
@@ -309,7 +309,7 @@
     <t>MOUSSAVOU Orphe Tresor</t>
   </si>
   <si>
-    <t>tresor.moussavou@anbg.ga</t>
+    <t>t.moussavou.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chauffeur DG</t>
@@ -321,7 +321,7 @@
     <t>ADAN-GBLENOU Loick Eklu Gagnon</t>
   </si>
   <si>
-    <t>loick.adan@anbg.ga</t>
+    <t>l.adan.anbg@gmail.com</t>
   </si>
   <si>
     <t>Conseiller Technique</t>
@@ -330,7 +330,7 @@
     <t>ATSAKOUNA Judicael</t>
   </si>
   <si>
-    <t>judicael.atsakouna@anbg.ga</t>
+    <t>j.atsakouna.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chargé d'étude</t>
@@ -339,7 +339,7 @@
     <t>EVOUNA OBAME Serge</t>
   </si>
   <si>
-    <t>serge.evouna@anbg.ga</t>
+    <t>s.evouna.anbg@gmail.com</t>
   </si>
   <si>
     <t>Assistant administratif</t>
@@ -348,7 +348,7 @@
     <t>KANGA Monique</t>
   </si>
   <si>
-    <t>monique.kanga@anbg.ga</t>
+    <t>m.kanga.anbg@gmail.com</t>
   </si>
   <si>
     <t>DGA</t>
@@ -363,19 +363,19 @@
     <t>LEYOGHO MAYILA Clif Loic</t>
   </si>
   <si>
-    <t>clif.leyogho@anbg.ga</t>
+    <t>c.leyogho.anbg@gmail.com</t>
   </si>
   <si>
     <t>MABADY BEHOBE Dick-Daniel</t>
   </si>
   <si>
-    <t>dick.mabady@anbg.ga</t>
+    <t>d.mabady.anbg@gmail.com</t>
   </si>
   <si>
     <t>MAYAGUI MANAMY Gilles</t>
   </si>
   <si>
-    <t>gilles.mayagui@anbg.ga</t>
+    <t>g.mayagui.anbg@gmail.com</t>
   </si>
   <si>
     <t>Attaché de cabinet</t>
@@ -384,19 +384,19 @@
     <t>MBAZOGO ELLA Urielle</t>
   </si>
   <si>
-    <t>urielle.mbazogo@anbg.ga</t>
+    <t>u.mbazogo.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOMBO Stecy Michel</t>
   </si>
   <si>
-    <t>stecy.mombo@anbg.ga</t>
+    <t>s.mombo.anbg@gmail.com</t>
   </si>
   <si>
     <t>NGUEMA Nadia Pascale</t>
   </si>
   <si>
-    <t>nadia.nguema@anbg.ga</t>
+    <t>n.nguema.anbg@gmail.com</t>
   </si>
   <si>
     <t>Secrétaire DG</t>
@@ -405,13 +405,13 @@
     <t>NTSAGA LEKELE Maureen</t>
   </si>
   <si>
-    <t>maureen.ntsaga@anbg.ga</t>
+    <t>m.ntsaga.anbg@gmail.com</t>
   </si>
   <si>
     <t>SIBHA NZE NZONG Ornelia</t>
   </si>
   <si>
-    <t>ornelia.sibha@anbg.ga</t>
+    <t>o.sibha.anbg@gmail.com</t>
   </si>
   <si>
     <t>À compléter</t>
@@ -426,7 +426,7 @@
     <t>ANGUE ALADE Kassirath</t>
   </si>
   <si>
-    <t>kassirath.angue@anbg.ga</t>
+    <t>k.angue.anbg@gmail.com</t>
   </si>
   <si>
     <t>SCIQ</t>
@@ -444,7 +444,7 @@
     <t>DOGUI Marie Raphaelle</t>
   </si>
   <si>
-    <t>raphaelle.dogui@anbg.ga</t>
+    <t>r.dogui.anbg@gmail.com</t>
   </si>
   <si>
     <t>DS</t>
@@ -459,7 +459,7 @@
     <t>KOMBA Joelle</t>
   </si>
   <si>
-    <t>joelle.komba@anbg.ga</t>
+    <t>j.komba.anbg@gmail.com</t>
   </si>
   <si>
     <t>Partenariats</t>
@@ -468,7 +468,7 @@
     <t>LEANDRY MBIRA</t>
   </si>
   <si>
-    <t>leandry.mbira@anbg.ga</t>
+    <t>l.mbira.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chargé statistiques</t>
@@ -477,13 +477,13 @@
     <t>MOUELLE MASSALA NDONGO Aaron</t>
   </si>
   <si>
-    <t>aaron.mouelle@anbg.ga</t>
+    <t>a.mouelle.anbg@gmail.com</t>
   </si>
   <si>
     <t>NDOUTOUME Jean Servais</t>
   </si>
   <si>
-    <t>servais.ndoutoume@anbg.ga</t>
+    <t>s.ndoutoume.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chef service Planification</t>
@@ -492,13 +492,13 @@
     <t>NGUEBET MOGOULA Hilaire</t>
   </si>
   <si>
-    <t>hilaire.nguebet@anbg.ga</t>
+    <t>h.nguebet.anbg@gmail.com</t>
   </si>
   <si>
     <t>NTSITSIGUI Yannis</t>
   </si>
   <si>
-    <t>yannis.ntsitsigui@anbg.ga</t>
+    <t>y.ntsitsigui.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chargé suivi académique</t>
@@ -516,7 +516,7 @@
     <t>AZIZET AKEWA Claude</t>
   </si>
   <si>
-    <t>claude.azizet@anbg.ga</t>
+    <t>c.azizet.anbg@gmail.com</t>
   </si>
   <si>
     <t>EB</t>
@@ -525,7 +525,7 @@
     <t>BISSONGUI MAKITA Raissa</t>
   </si>
   <si>
-    <t>raissa.bissongui@anbg.ga</t>
+    <t>r.bissongui.anbg@gmail.com</t>
   </si>
   <si>
     <t>Gestionnaire senior</t>
@@ -534,67 +534,67 @@
     <t>LEKA Noeline</t>
   </si>
   <si>
-    <t>noeline.leka@anbg.ga</t>
+    <t>n.leka.anbg@gmail.com</t>
   </si>
   <si>
     <t>LEMBA Sigrid</t>
   </si>
   <si>
-    <t>sigrid.lemba@anbg.ga</t>
+    <t>s.lemba.anbg@gmail.com</t>
   </si>
   <si>
     <t>MAKANGOU Zita</t>
   </si>
   <si>
-    <t>zita.makangou@anbg.ga</t>
+    <t>z.makangou.anbg@gmail.com</t>
   </si>
   <si>
     <t>MAVIOGA Leger</t>
   </si>
   <si>
-    <t>leger.mavioga@anbg.ga</t>
+    <t>l.mavioga.anbg@gmail.com</t>
   </si>
   <si>
     <t>MENDOME Nadine</t>
   </si>
   <si>
-    <t>nadine.mendome@anbg.ga</t>
+    <t>n.mendome.anbg@gmail.com</t>
   </si>
   <si>
     <t>MOUKAGNI Estelle</t>
   </si>
   <si>
-    <t>estelle.moukagni@anbg.ga</t>
+    <t>e.moukagni.anbg@gmail.com</t>
   </si>
   <si>
     <t>NGOUBILI Lidy</t>
   </si>
   <si>
-    <t>lidy.ngoubili@anbg.ga</t>
+    <t>l.ngoubili.anbg@gmail.com</t>
   </si>
   <si>
     <t>NKOURA Charly</t>
   </si>
   <si>
-    <t>charly.nkoura@anbg.ga</t>
+    <t>c.nkoura.anbg@gmail.com</t>
   </si>
   <si>
     <t>NYANGUI Sandrine</t>
   </si>
   <si>
-    <t>sandrine.nyangui@anbg.ga</t>
+    <t>s.nyangui.anbg@gmail.com</t>
   </si>
   <si>
     <t>SIMBOU Laurencienne</t>
   </si>
   <si>
-    <t>laurencienne.simbou@anbg.ga</t>
+    <t>l.simbou.anbg@gmail.com</t>
   </si>
   <si>
     <t>MAGNANGANI ERIMI Belinda</t>
   </si>
   <si>
-    <t>belinda.magnangani@anbg.ga</t>
+    <t>b.magnangani.anbg@gmail.com</t>
   </si>
   <si>
     <t>Chef service EB</t>
@@ -603,7 +603,7 @@
     <t>MENOUETON Codjo</t>
   </si>
   <si>
-    <t>codjo.menoueton@anbg.ga</t>
+    <t>c.menoueton.anbg@gmail.com</t>
   </si>
   <si>
     <t>Responsable pôle</t>
@@ -612,7 +612,7 @@
     <t>TOUNGOU Carine</t>
   </si>
   <si>
-    <t>carine.toungou@anbg.ga</t>
+    <t>c.toungou.anbg@gmail.com</t>
   </si>
   <si>
     <t>Responsable pôle étranger</t>
@@ -621,7 +621,7 @@
     <t>SIMBA Marie Louise</t>
   </si>
   <si>
-    <t>marie.simba@anbg.ga</t>
+    <t>m.simba.anbg@gmail.com</t>
   </si>
   <si>
     <t>ENB</t>
@@ -645,7 +645,7 @@
     <t>MBAZOO Christel</t>
   </si>
   <si>
-    <t>christel.mbazoo@anbg.ga</t>
+    <t>c.mbazoo.anbg@gmail.com</t>
   </si>
   <si>
     <t>CRP</t>
@@ -657,19 +657,19 @@
     <t>NGOMA Lucrecia</t>
   </si>
   <si>
-    <t>lucrecia.ngoma@anbg.ga</t>
+    <t>l.ngoma.anbg@gmail.com</t>
   </si>
   <si>
     <t>OSSI Hans</t>
   </si>
   <si>
-    <t>hans.ossi@anbg.ga</t>
+    <t>h.ossi.anbg@gmail.com</t>
   </si>
   <si>
     <t>MBOUMBA Noelle</t>
   </si>
   <si>
-    <t>noelle.mboumba@anbg.ga</t>
+    <t>n.mboumba.anbg@gmail.com</t>
   </si>
   <si>
     <t>Responsable communication</t>
@@ -678,13 +678,13 @@
     <t>YEMBI Marvin</t>
   </si>
   <si>
-    <t>marvin.yembi@anbg.ga</t>
+    <t>m.yembi.anbg@gmail.com</t>
   </si>
   <si>
     <t>LEYIGUI Wilfried</t>
   </si>
   <si>
-    <t>wilfried.leyigui@anbg.ga</t>
+    <t>w.leyigui.anbg@gmail.com</t>
   </si>
   <si>
     <t>GDS</t>
@@ -696,19 +696,19 @@
     <t>MAGNET Clovis</t>
   </si>
   <si>
-    <t>clovis.magnet@anbg.ga</t>
+    <t>c.magnet.anbg@gmail.com</t>
   </si>
   <si>
     <t>KOMBA Staelle</t>
   </si>
   <si>
-    <t>staelle.komba@anbg.ga</t>
+    <t>s.komba.anbg@gmail.com</t>
   </si>
   <si>
     <t>CAMARA François</t>
   </si>
   <si>
-    <t>francois.camara@anbg.ga</t>
+    <t>f.camara.anbg@gmail.com</t>
   </si>
   <si>
     <t>SIRS</t>
@@ -720,25 +720,25 @@
     <t>EBINDA Roger</t>
   </si>
   <si>
-    <t>roger.ebinda@anbg.ga</t>
+    <t>r.ebinda.anbg@gmail.com</t>
   </si>
   <si>
     <t>NGUEMEDZANG Renaud</t>
   </si>
   <si>
-    <t>renaud.nguemedzang@anbg.ga</t>
+    <t>r.nguemedzang.anbg@gmail.com</t>
   </si>
   <si>
     <t>OSSA Charles</t>
   </si>
   <si>
-    <t>charles.ossa@anbg.ga</t>
+    <t>c.ossa.anbg@gmail.com</t>
   </si>
   <si>
     <t>Arnold MINDZELI</t>
   </si>
   <si>
-    <t>arnold.mindzeli@anbg.ga</t>
+    <t>a.mindzeli.anbg@gmail.com</t>
   </si>
   <si>
     <t>Service / unité</t>

</xml_diff>